<commit_message>
fix(providers): record wechat withdrawal fees and correct example configs
- Example statements for ccb_debit and pab_debit are written with
  two-decimal text cells, as the banks export them, so the golden output
  and balance assertions carry two decimals.
- Add a generic fee posting: a provider sets Transaction.fee and the
  writer posts it to providers.<id>.fee_account, then defaults.fee_account
  (default Expenses:FIXME). A WeChat withdrawal with a service fee now
  takes the gross amount from the wallet and credits the bank net of the
  fee.
- bean-sieve.example.yaml maps the app_store Apple ID to an Assets
  account, points every zabank_debit currency at one account, and drops
  the no-op balance flag from welab_debit; provider pages explain why.

Refs: APP-276
</commit_message>
<xml_diff>
--- a/examples/pab_debit/平安银行借记卡流水.xlsx
+++ b/examples/pab_debit/平安银行借记卡流水.xlsx
@@ -511,11 +511,15 @@
           <t>转入</t>
         </is>
       </c>
-      <c r="G3" t="n">
-        <v>7500</v>
-      </c>
-      <c r="H3" t="n">
-        <v>7500</v>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>7500.00</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>7500.00</t>
+        </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -564,11 +568,15 @@
           <t>转出</t>
         </is>
       </c>
-      <c r="G4" t="n">
-        <v>33</v>
-      </c>
-      <c r="H4" t="n">
-        <v>7467</v>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>33.00</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>7467.00</t>
+        </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -617,11 +625,15 @@
           <t>转出</t>
         </is>
       </c>
-      <c r="G5" t="n">
-        <v>288</v>
-      </c>
-      <c r="H5" t="n">
-        <v>7179</v>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>288.00</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>7179.00</t>
+        </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -670,11 +682,15 @@
           <t>转出</t>
         </is>
       </c>
-      <c r="G6" t="n">
-        <v>2000</v>
-      </c>
-      <c r="H6" t="n">
-        <v>5179</v>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2000.00</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>5179.00</t>
+        </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -719,11 +735,15 @@
           <t>转入</t>
         </is>
       </c>
-      <c r="G7" t="n">
-        <v>88</v>
-      </c>
-      <c r="H7" t="n">
-        <v>5267</v>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>88.00</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>5267.00</t>
+        </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -768,11 +788,15 @@
           <t>转入</t>
         </is>
       </c>
-      <c r="G8" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="H8" t="n">
-        <v>5268.3</v>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>1.30</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>5268.30</t>
+        </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -821,11 +845,15 @@
           <t>转出</t>
         </is>
       </c>
-      <c r="G9" t="n">
-        <v>24</v>
-      </c>
-      <c r="H9" t="n">
-        <v>5244.3</v>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>24.00</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>5244.30</t>
+        </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>

</xml_diff>